<commit_message>
adds build/www for dereferencable ttl, rdf+xml and json-ld for all concepts
</commit_message>
<xml_diff>
--- a/classification-systems/nzlum/build/commodities.xlsx
+++ b/classification-systems/nzlum/build/commodities.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Collections" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collections" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3057,7 +3057,11 @@
           <t>Pulses</t>
         </is>
       </c>
-      <c r="B202" s="2" t="inlineStr"/>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>azuki bean</t>
+        </is>
+      </c>
       <c r="C202" s="2" t="inlineStr"/>
       <c r="D202" s="2" t="inlineStr"/>
       <c r="E202" s="2" t="inlineStr"/>
@@ -3067,7 +3071,7 @@
       <c r="A203" s="2" t="n"/>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>azuki bean</t>
+          <t>broad beans</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr"/>
@@ -3079,7 +3083,7 @@
       <c r="A204" s="2" t="n"/>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>broad beans</t>
+          <t>chickpeas</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr"/>
@@ -3091,7 +3095,7 @@
       <c r="A205" s="2" t="n"/>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>chickpeas</t>
+          <t>cowpea</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr"/>
@@ -3103,7 +3107,7 @@
       <c r="A206" s="2" t="n"/>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>cowpea</t>
+          <t>field beans</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr"/>
@@ -3115,7 +3119,7 @@
       <c r="A207" s="2" t="n"/>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>field beans</t>
+          <t>field peas</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr"/>
@@ -3127,7 +3131,7 @@
       <c r="A208" s="2" t="n"/>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>field peas</t>
+          <t>lentils</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr"/>
@@ -3139,7 +3143,7 @@
       <c r="A209" s="2" t="n"/>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>lentils</t>
+          <t>lupins</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr"/>
@@ -3151,7 +3155,7 @@
       <c r="A210" s="2" t="n"/>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>lupins</t>
+          <t>mung bean</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr"/>
@@ -4017,18 +4021,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A2:A33"/>
+    <mergeCell ref="A34:A45"/>
+    <mergeCell ref="A46:A64"/>
+    <mergeCell ref="A65:A79"/>
+    <mergeCell ref="A80:A89"/>
+    <mergeCell ref="A90:A152"/>
+    <mergeCell ref="A154:A176"/>
     <mergeCell ref="A177:A186"/>
-    <mergeCell ref="A34:A45"/>
-    <mergeCell ref="A65:A79"/>
-    <mergeCell ref="A214:A281"/>
-    <mergeCell ref="A154:A176"/>
-    <mergeCell ref="A2:A33"/>
+    <mergeCell ref="A187:A195"/>
     <mergeCell ref="A196:A201"/>
     <mergeCell ref="A202:A213"/>
-    <mergeCell ref="A187:A195"/>
-    <mergeCell ref="A46:A64"/>
-    <mergeCell ref="A90:A152"/>
-    <mergeCell ref="A80:A89"/>
+    <mergeCell ref="A214:A281"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>